<commit_message>
Add Diversification & Variance PDF/Excel from all course materials
- Screenshots from Sample Q22, Mock Q29, and Ch.9 lecture slides
- Excel workbook with embedded PDF tab (like Labor-Leisure)
- Study Tracker Diversification row links to embedded PDF tab
- Source audit: no div/var problems in HW1, HW2, or Sample Ch.4

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Study_Tracker.xlsx
+++ b/Study_Tracker.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labor-Leisure PDF" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diversification PDF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -112,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,6 +139,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +230,236 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>128</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>192</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>255</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>319</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>383</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>446</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>510</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1019,71 +1253,75 @@
           <t>— Not yet</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Still need to practice</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr"/>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Also: full Div/Var workbook (online)</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Go to embedded PDF tab</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Ch. 4 Total</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="A15" s="13" t="n"/>
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Ch. 9 Total</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n"/>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Green = reviewed / done</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Not green = still need practice</t>
         </is>
@@ -1096,6 +1334,8 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1114,7 +1354,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="105" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
         </is>

</xml_diff>

<commit_message>
Add Marginal Utility guide PDF/Excel with increasing MU example
Explains TU, MU (first derivative), and second derivative with the user's
example: MU at unit 1 = 10 and at unit 2 = 20 means increasing MU and
risk-loving preferences. Embedded in Excel and linked from Risk Attitudes row.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Study_Tracker.xlsx
+++ b/Study_Tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labor-Leisure PDF" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diversification PDF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marginal Utility PDF" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -113,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -132,6 +133,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -676,6 +680,161 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>128</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>192</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>255</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>319</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1209,8 +1368,16 @@
           <t>✓ Done</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Also: full MU guide workbook (online)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Go to embedded PDF tab</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1235,93 +1402,93 @@
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Ch. 9</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Diversification</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>— Not yet</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>Also: full Div/Var workbook (online)</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Go to embedded PDF tab</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Ch. 4 Total</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Ch. 9 Total</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Green = reviewed / done</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Not green = still need practice</t>
         </is>
@@ -1334,8 +1501,10 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1354,7 +1523,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
         </is>
@@ -1379,7 +1548,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="105" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
         </is>

</xml_diff>